<commit_message>
trying to get a way to add translation to [Translation Missing] entries
Signed-off-by: look-luc <denardiluc@gmail.com>
</commit_message>
<xml_diff>
--- a/data/tooro/lit_tooro_random_15.xlsx
+++ b/data/tooro/lit_tooro_random_15.xlsx
@@ -1,17 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10628"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucdenardi/Desktop/code_lang/python/East-African-Dataset/data/tooro/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F13F6F3-ECAC-7C4F-86CF-D5DD8972BD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="lit_tooro_random_15" sheetId="1" r:id="rId5"/>
+    <sheet name="lit_tooro_random_15" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="310" uniqueCount="137">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="317" uniqueCount="144">
   <si>
     <t>Unnamed: 0</t>
   </si>
@@ -422,22 +431,45 @@
   </si>
   <si>
     <t>nabariho nib-o babarw-a</t>
+  </si>
+  <si>
+    <t>The power abused your mom your presence.</t>
+  </si>
+  <si>
+    <t>Skins your honor __(3rd singular) feathers obstruct your __(past, reciprocal, 3rd plural) __(singular) __(present)</t>
+  </si>
+  <si>
+    <t>Usually advice, not ignore child's</t>
+  </si>
+  <si>
+    <t>___(V.PRS.PROG.3.SG) ___(PST.PFR.2.SG)-__ house your(pl) ___(V.PST.REC.2.SG)</t>
+  </si>
+  <si>
+    <t>___(N.SG.N1) ___(NSG.N1) becomes ____</t>
+  </si>
+  <si>
+    <t>___ prs.___ ___.pst ___.sg.n14 ___</t>
+  </si>
+  <si>
+    <t>animals/abstract it becomes  your sg.n14-___ ___.sg.n14</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -446,40 +478,43 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -669,20 +704,26 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:K41"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
-    <col customWidth="1" min="9" max="9" width="87.13"/>
+    <col min="3" max="3" width="30.6640625" customWidth="1"/>
+    <col min="6" max="6" width="88.83203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="69.1640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="87.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
@@ -714,12 +755,12 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A2" s="1">
-        <v>12560.0</v>
+        <v>12560</v>
       </c>
       <c r="B2" s="1">
-        <v>77893.0</v>
+        <v>77893</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>10</v>
@@ -745,13 +786,16 @@
       <c r="J2" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="3">
+      <c r="K2" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A3" s="1">
-        <v>38416.0</v>
+        <v>38416</v>
       </c>
       <c r="B3" s="1">
-        <v>228758.0</v>
+        <v>228758</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>18</v>
@@ -777,13 +821,16 @@
       <c r="J3" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="4">
+      <c r="K3" s="1" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A4" s="1">
-        <v>6732.0</v>
+        <v>6732</v>
       </c>
       <c r="B4" s="1">
-        <v>40667.0</v>
+        <v>40667</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>22</v>
@@ -809,13 +856,16 @@
       <c r="J4" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="5">
+      <c r="K4" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A5" s="1">
-        <v>40233.0</v>
+        <v>40233</v>
       </c>
       <c r="B5" s="1">
-        <v>240424.0</v>
+        <v>240424</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>26</v>
@@ -841,13 +891,16 @@
       <c r="J5" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="6">
+      <c r="K5" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A6" s="1">
-        <v>2956.0</v>
+        <v>2956</v>
       </c>
       <c r="B6" s="1">
-        <v>18150.0</v>
+        <v>18150</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>30</v>
@@ -873,13 +926,16 @@
       <c r="J6" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="7">
+      <c r="K6" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A7" s="1">
-        <v>17783.0</v>
+        <v>17783</v>
       </c>
       <c r="B7" s="1">
-        <v>102959.0</v>
+        <v>102959</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>34</v>
@@ -905,13 +961,16 @@
       <c r="J7" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="8">
+      <c r="K7" s="1" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A8" s="1">
-        <v>2945.0</v>
+        <v>2945</v>
       </c>
       <c r="B8" s="1">
-        <v>18139.0</v>
+        <v>18139</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>30</v>
@@ -937,13 +996,16 @@
       <c r="J8" s="1" t="s">
         <v>17</v>
       </c>
-    </row>
-    <row r="9">
+      <c r="K8" s="1" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A9" s="1">
-        <v>35633.0</v>
+        <v>35633</v>
       </c>
       <c r="B9" s="1">
-        <v>211379.0</v>
+        <v>211379</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>41</v>
@@ -970,12 +1032,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A10" s="1">
-        <v>35671.0</v>
+        <v>35671</v>
       </c>
       <c r="B10" s="1">
-        <v>211417.0</v>
+        <v>211417</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>41</v>
@@ -1002,12 +1064,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A11" s="1">
-        <v>17749.0</v>
+        <v>17749</v>
       </c>
       <c r="B11" s="1">
-        <v>102925.0</v>
+        <v>102925</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>34</v>
@@ -1034,12 +1096,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A12" s="1">
-        <v>12581.0</v>
+        <v>12581</v>
       </c>
       <c r="B12" s="1">
-        <v>77914.0</v>
+        <v>77914</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>10</v>
@@ -1066,12 +1128,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A13" s="1">
-        <v>40276.0</v>
+        <v>40276</v>
       </c>
       <c r="B13" s="1">
-        <v>240467.0</v>
+        <v>240467</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>26</v>
@@ -1098,12 +1160,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A14" s="1">
-        <v>38423.0</v>
+        <v>38423</v>
       </c>
       <c r="B14" s="1">
-        <v>228765.0</v>
+        <v>228765</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>18</v>
@@ -1130,12 +1192,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A15" s="1">
-        <v>14213.0</v>
+        <v>14213</v>
       </c>
       <c r="B15" s="1">
-        <v>84693.0</v>
+        <v>84693</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>34</v>
@@ -1162,12 +1224,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A16" s="1">
-        <v>38373.0</v>
+        <v>38373</v>
       </c>
       <c r="B16" s="1">
-        <v>228715.0</v>
+        <v>228715</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>18</v>
@@ -1194,12 +1256,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A17" s="1">
-        <v>26155.0</v>
+        <v>26155</v>
       </c>
       <c r="B17" s="1">
-        <v>151964.0</v>
+        <v>151964</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>63</v>
@@ -1226,12 +1288,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A18" s="1">
-        <v>10669.0</v>
+        <v>10669</v>
       </c>
       <c r="B18" s="1">
-        <v>64447.0</v>
+        <v>64447</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>64</v>
@@ -1258,12 +1320,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A19" s="1">
-        <v>1821.0</v>
+        <v>1821</v>
       </c>
       <c r="B19" s="1">
-        <v>12421.0</v>
+        <v>12421</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>68</v>
@@ -1290,12 +1352,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A20" s="1">
-        <v>14253.0</v>
+        <v>14253</v>
       </c>
       <c r="B20" s="1">
-        <v>84733.0</v>
+        <v>84733</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>34</v>
@@ -1322,12 +1384,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A21" s="1">
-        <v>38358.0</v>
+        <v>38358</v>
       </c>
       <c r="B21" s="1">
-        <v>228700.0</v>
+        <v>228700</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>18</v>
@@ -1354,12 +1416,12 @@
         <v>17</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A22" s="1">
-        <v>16091.0</v>
+        <v>16091</v>
       </c>
       <c r="B22" s="1">
-        <v>95920.0</v>
+        <v>95920</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>10</v>
@@ -1383,12 +1445,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A23" s="1">
-        <v>17718.0</v>
+        <v>17718</v>
       </c>
       <c r="B23" s="1">
-        <v>102894.0</v>
+        <v>102894</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>34</v>
@@ -1412,12 +1474,12 @@
         <v>83</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A24" s="1">
-        <v>24864.0</v>
+        <v>24864</v>
       </c>
       <c r="B24" s="1">
-        <v>144325.0</v>
+        <v>144325</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>84</v>
@@ -1441,12 +1503,12 @@
         <v>87</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A25" s="1">
-        <v>35721.0</v>
+        <v>35721</v>
       </c>
       <c r="B25" s="1">
-        <v>211467.0</v>
+        <v>211467</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>41</v>
@@ -1470,12 +1532,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A26" s="1">
-        <v>38374.0</v>
+        <v>38374</v>
       </c>
       <c r="B26" s="1">
-        <v>228716.0</v>
+        <v>228716</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>18</v>
@@ -1499,12 +1561,12 @@
         <v>93</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A27" s="1">
-        <v>10670.0</v>
+        <v>10670</v>
       </c>
       <c r="B27" s="1">
-        <v>64448.0</v>
+        <v>64448</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>64</v>
@@ -1528,12 +1590,12 @@
         <v>96</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A28" s="1">
-        <v>6667.0</v>
+        <v>6667</v>
       </c>
       <c r="B28" s="1">
-        <v>40602.0</v>
+        <v>40602</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>22</v>
@@ -1557,12 +1619,12 @@
         <v>99</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A29" s="1">
-        <v>38438.0</v>
+        <v>38438</v>
       </c>
       <c r="B29" s="1">
-        <v>228780.0</v>
+        <v>228780</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>18</v>
@@ -1586,12 +1648,12 @@
         <v>102</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A30" s="1">
-        <v>40314.0</v>
+        <v>40314</v>
       </c>
       <c r="B30" s="1">
-        <v>240505.0</v>
+        <v>240505</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>26</v>
@@ -1615,12 +1677,12 @@
         <v>105</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A31" s="1">
-        <v>2950.0</v>
+        <v>2950</v>
       </c>
       <c r="B31" s="1">
-        <v>18144.0</v>
+        <v>18144</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>30</v>
@@ -1644,12 +1706,12 @@
         <v>108</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A32" s="1">
-        <v>10662.0</v>
+        <v>10662</v>
       </c>
       <c r="B32" s="1">
-        <v>64440.0</v>
+        <v>64440</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>64</v>
@@ -1673,12 +1735,12 @@
         <v>111</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A33" s="1">
-        <v>31670.0</v>
+        <v>31670</v>
       </c>
       <c r="B33" s="1">
-        <v>186874.0</v>
+        <v>186874</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>112</v>
@@ -1702,12 +1764,12 @@
         <v>115</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A34" s="1">
-        <v>16121.0</v>
+        <v>16121</v>
       </c>
       <c r="B34" s="1">
-        <v>95950.0</v>
+        <v>95950</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>10</v>
@@ -1731,12 +1793,12 @@
         <v>118</v>
       </c>
     </row>
-    <row r="35">
+    <row r="35" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A35" s="1">
-        <v>16120.0</v>
+        <v>16120</v>
       </c>
       <c r="B35" s="1">
-        <v>95949.0</v>
+        <v>95949</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>10</v>
@@ -1760,12 +1822,12 @@
         <v>121</v>
       </c>
     </row>
-    <row r="36">
+    <row r="36" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A36" s="1">
-        <v>12583.0</v>
+        <v>12583</v>
       </c>
       <c r="B36" s="1">
-        <v>77916.0</v>
+        <v>77916</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>10</v>
@@ -1789,12 +1851,12 @@
         <v>124</v>
       </c>
     </row>
-    <row r="37">
+    <row r="37" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="1">
-        <v>16055.0</v>
+        <v>16055</v>
       </c>
       <c r="B37" s="1">
-        <v>95884.0</v>
+        <v>95884</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>10</v>
@@ -1818,12 +1880,12 @@
         <v>127</v>
       </c>
     </row>
-    <row r="38">
+    <row r="38" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="1">
-        <v>1817.0</v>
+        <v>1817</v>
       </c>
       <c r="B38" s="1">
-        <v>12417.0</v>
+        <v>12417</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>68</v>
@@ -1847,12 +1909,12 @@
         <v>130</v>
       </c>
     </row>
-    <row r="39">
+    <row r="39" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="1">
-        <v>2985.0</v>
+        <v>2985</v>
       </c>
       <c r="B39" s="1">
-        <v>18179.0</v>
+        <v>18179</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>30</v>
@@ -1876,12 +1938,12 @@
         <v>133</v>
       </c>
     </row>
-    <row r="40">
+    <row r="40" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="1">
-        <v>16104.0</v>
+        <v>16104</v>
       </c>
       <c r="B40" s="1">
-        <v>95933.0</v>
+        <v>95933</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>10</v>
@@ -1905,12 +1967,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="41">
+    <row r="41" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="1">
-        <v>6690.0</v>
+        <v>6690</v>
       </c>
       <c r="B41" s="1">
-        <v>40625.0</v>
+        <v>40625</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>22</v>
@@ -1935,6 +1997,6 @@
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
trying to fix wrong translation
Signed-off-by: look-luc <denardiluc@gmail.com>
</commit_message>
<xml_diff>
--- a/data/tooro/lit_tooro_random_15.xlsx
+++ b/data/tooro/lit_tooro_random_15.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucdenardi/Desktop/code_lang/python/East-African-Dataset/data/tooro/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F13F6F3-ECAC-7C4F-86CF-D5DD8972BD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10DE9BD1-E5A5-B34A-8DF5-208163B917A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -442,9 +442,6 @@
     <t>Usually advice, not ignore child's</t>
   </si>
   <si>
-    <t>___(V.PRS.PROG.3.SG) ___(PST.PFR.2.SG)-__ house your(pl) ___(V.PST.REC.2.SG)</t>
-  </si>
-  <si>
     <t>___(N.SG.N1) ___(NSG.N1) becomes ____</t>
   </si>
   <si>
@@ -452,6 +449,9 @@
   </si>
   <si>
     <t>animals/abstract it becomes  your sg.n14-___ ___.sg.n14</t>
+  </si>
+  <si>
+    <t>requesting swept house own before not say pl.n1.pss.n9-___ prs.hab.2.sg-___</t>
   </si>
 </sst>
 </file>
@@ -892,7 +892,7 @@
         <v>17</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -927,7 +927,7 @@
         <v>17</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -962,7 +962,7 @@
         <v>17</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
@@ -997,7 +997,7 @@
         <v>17</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="9" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">

</xml_diff>